<commit_message>
Verificación de creador y restricciones para Operador
</commit_message>
<xml_diff>
--- a/public/plantilla_importacion_productos.xlsx
+++ b/public/plantilla_importacion_productos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS VIVOBOOK\Documents\Programación\Angular\optica-angular\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1F1919B-5CC9-4D97-B029-7A17545780A9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7482A92-4DAF-4D62-BFB7-BFE38B0B666A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{09DB8C61-75D7-4791-8621-EFA47FDED1E7}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="18105" xr2:uid="{09DB8C61-75D7-4791-8621-EFA47FDED1E7}"/>
   </bookViews>
   <sheets>
     <sheet name="ECUPERSA ACADEMIC" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t xml:space="preserve">PLANTILLA DE PRODUCTOS </t>
   </si>
@@ -82,6 +82,9 @@
   </si>
   <si>
     <t>COSTO</t>
+  </si>
+  <si>
+    <t>GRUPO</t>
   </si>
 </sst>
 </file>
@@ -586,7 +589,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0451375-9663-48E4-A3F1-D88552ABDB00}">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -596,7 +599,7 @@
     <col min="5" max="5" width="33.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="11" t="s">
         <v>14</v>
       </c>
@@ -605,9 +608,10 @@
       <c r="D1" s="12"/>
       <c r="E1" s="13"/>
       <c r="F1" s="9"/>
-      <c r="G1" s="1"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>0</v>
       </c>
@@ -616,9 +620,10 @@
       <c r="D2" s="15"/>
       <c r="E2" s="16"/>
       <c r="F2" s="10"/>
-      <c r="G2" s="1"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="1"/>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>1</v>
       </c>
@@ -629,11 +634,14 @@
       <c r="D3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="2"/>
+      <c r="E3" s="2" t="s">
+        <v>11</v>
+      </c>
       <c r="F3" s="2"/>
-      <c r="G3" s="4"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="4"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="19" t="s">
         <v>3</v>
       </c>
@@ -644,13 +652,12 @@
       <c r="D4" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="6" t="s">
-        <v>11</v>
-      </c>
+      <c r="E4" s="6"/>
       <c r="F4" s="6"/>
-      <c r="G4" s="4"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="1:7" ht="38.25" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" ht="38.25" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>5</v>
       </c>
@@ -667,9 +674,12 @@
         <v>8</v>
       </c>
       <c r="F5" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="8" t="s">
+      <c r="H5" s="8" t="s">
         <v>9</v>
       </c>
     </row>

</xml_diff>